<commit_message>
Agregar copas de la foto 2 y lista de dudas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -1057,7 +1057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1066,9 +1066,11 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1089,30 +1091,40 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Medida (℅)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Pie</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Nota en lápiz</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1126,24 +1138,30 @@
       </c>
       <c r="B2" s="2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n">
         <v>320</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="F2" s="2" t="n">
         <v>450</v>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Requem. 8</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Prensa</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="J2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>En lápiz: "Requem. 8" y un "300" debajo del B:450 (¿B corregido a 300?)</t>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Hay un "300" en lápiz debajo del B:450 (¿B corregido a 300?). ¿Qué es "Requem. 8"?</t>
         </is>
       </c>
     </row>
@@ -1155,22 +1173,565 @@
       </c>
       <c r="B3" s="3" t="inlineStr"/>
       <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="n">
         <v>570</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="F3" s="3" t="n">
         <v>250</v>
       </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Prensa</t>
         </is>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="J3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="I3" s="3" t="inlineStr"/>
+      <c r="K3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Copa Romina Vino</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>15,3</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Lorena V.B</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Copa Presidente Champ</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Copa Clarito Inés De los Santos</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Presi V.T</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Copa Prince Agua</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>19,7</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>London 98</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>El peso está remarcado/sobrescrito: confirmar que es 220</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Copa Barón</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>London 98</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Copa Chandón 2021</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>London 98</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>El pie no está escrito: hay comillas (") debajo de "Pie London 98" de la fila de arriba</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Copa Magnífica</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Delise</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Copa Venus Champ</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Copa Flavia Champ</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Copa Ceci Flauta</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>170</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Presi Agua</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Copa Him-Chan Agua</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Venus V.B</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Copa Retro</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Mod II Agua</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Copa Premium Mediana</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Mini Marisco</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Copa Premium Chica</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Mod II Agua</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Copa Silvia Agua</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Silvia Agua</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mover las copas de Prensa a una pestaña PRENSA propia
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -18,7 +18,7 @@
     <sheet name="TAPA" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="JARRA" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="ACEITERA" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="OTROS" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="PRENSA" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -94,10 +94,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -651,7 +651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -707,47 +707,47 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Plato</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Plato Pizza</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="3" t="n">
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="E2" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Prensa</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="3" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Faro</t>
+          <t>Copa</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Faro Puma</t>
+          <t>Copa Alaska</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="n">
-        <v>130</v>
+        <v>320</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>450</v>
@@ -760,85 +760,85 @@
       <c r="G3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="3" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>En lápiz: "Requem. 8" y un "300" debajo del B:450 (¿B corregido a 300?)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Faro</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Faro Puma</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Prensa</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Faro</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Faro Ford</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="n">
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="n">
         <v>452</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E5" s="2" t="n">
         <v>600</v>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Prensa</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Filtro</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Filtro Nº 2</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="n">
-        <v>245</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>500</v>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Prensa</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Filtro</t>
+          <t>Copa</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Filtro Nº 4</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>SINAC</t>
-        </is>
-      </c>
+          <t>Copa Milk Shake</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="n">
-        <v>40</v>
+        <v>570</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>600</v>
+        <v>250</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -848,125 +848,121 @@
       <c r="G6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Filtro</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Filtro Nº 2</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="n">
+        <v>245</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Prensa</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Filtro</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Filtro Nº 4</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>SINAC</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Prensa</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Escrito en lápiz; "SINAC" con flecha desde B:600</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Base Velador</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Base Velador Grande</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="n">
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="n">
         <v>465</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E9" s="2" t="n">
         <v>400</v>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Prensa</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="G9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Base Velador</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Base Velador Chico</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Rococo</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>280</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>600</v>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Prensa</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>"Rococo" está escrito debajo del Chico</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Lupa</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Lupa Nº 3</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>FYW</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>88</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>500</v>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Prensa</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="3" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Lupa</t>
+          <t>Base Velador</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Lupa Nº 4</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr"/>
+          <t>Base Velador Chico</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Rococo</t>
+        </is>
+      </c>
       <c r="D10" s="3" t="n">
-        <v>350</v>
+        <v>280</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
@@ -976,29 +972,33 @@
       <c r="G10" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>"Rococo" está escrito debajo del Chico</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Vidrio</t>
+          <t>Lupa</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Vidrio</t>
+          <t>Lupa Nº 3</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>FYW</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>620</v>
+        <v>88</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1008,43 +1008,103 @@
       <c r="G11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Lupa</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Lupa Nº 4</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Prensa</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Vidrio</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Vidrio</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>620</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Prensa</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Escrito en lápiz</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Baliza</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Baliza Anillada Grande</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>BALIZAR</t>
         </is>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D14" s="2" t="n">
         <v>650</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E14" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Prensa</t>
         </is>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="G14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="3" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1057,7 +1117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1133,125 +1193,133 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Copa Alaska</t>
+          <t>Copa Romina Vino</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>15,3</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="n">
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>450</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Requem. 8</t>
-        </is>
-      </c>
+        <v>230</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Lorena V.B</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Prensa</t>
+          <t>Copas</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Hay un "300" en lápiz debajo del B:450 (¿B corregido a 300?). ¿Qué es "Requem. 8"?</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Copa Milk Shake</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr"/>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="n">
-        <v>570</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Prensa</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" s="3" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Copa Presidente Champ</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Copa Romina Vino</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr"/>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Pegada</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>15,3</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="n">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Copa Clarito Inés De los Santos</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Lorena V.B</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Presi V.T</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="J4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="3" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Copa Presidente Champ</t>
+          <t>Copa Prince Agua</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr"/>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>19,7</t>
+        </is>
+      </c>
       <c r="E5" s="3" t="n">
-        <v>180</v>
+        <v>220</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
+        <v>220</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>London 98</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
@@ -1260,125 +1328,129 @@
       <c r="J5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>El peso está remarcado/sobrescrito: confirmar que es 220</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Copa Clarito Inés De los Santos</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr"/>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="n">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Copa Barón</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F6" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>London 98</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Copa Chandón 2021</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="n">
         <v>230</v>
       </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Presi V.T</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="F7" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>London 98</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="J7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Copa Prince Agua</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Pegada</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>19,7</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>220</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>220</v>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>London 98</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>El pie no está escrito: hay comillas (") debajo de "Pie London 98" de la fila de arriba</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Copa Magnífica</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="n">
+        <v>160</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Delise</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>El peso está remarcado/sobrescrito: confirmar que es 220</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Copa Barón</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Estirada</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="n">
-        <v>250</v>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>London 98</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" s="3" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Copa Chandón 2021</t>
+          <t>Copa Venus Champ</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
@@ -1389,16 +1461,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="n">
-        <v>230</v>
+        <v>160</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>200</v>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>London 98</t>
-        </is>
-      </c>
+        <v>220</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1408,330 +1476,260 @@
       <c r="J9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>El pie no está escrito: hay comillas (") debajo de "Pie London 98" de la fila de arriba</t>
-        </is>
-      </c>
+      <c r="K9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Copa Magnífica</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr"/>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Copa Flavia Champ</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Estirada</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="n">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Copa Ceci Flauta</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="F11" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Delise</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Presi Agua</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J10" s="3" t="n">
+      <c r="J11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Copa Venus Champ</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr"/>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Estirada</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="n">
-        <v>160</v>
-      </c>
-      <c r="F11" s="3" t="n">
+      <c r="K11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Copa Him-Chan Agua</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Venus V.B</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Copa Retro</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="F13" s="2" t="n">
         <v>220</v>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Mod II Agua</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J11" s="3" t="n">
+      <c r="J13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Copa Flavia Champ</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Copa Premium Mediana</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Mini Marisco</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Copa Premium Chica</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Mod II Agua</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Copa Silvia Agua</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Silvia Agua</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Estirada</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="n">
-        <v>160</v>
-      </c>
-      <c r="F12" s="3" t="n">
-        <v>220</v>
-      </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J12" s="3" t="n">
+      <c r="J16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Copa Ceci Flauta</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr"/>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Estirada</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>170</v>
-      </c>
-      <c r="F13" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Presi Agua</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Copa Him-Chan Agua</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr"/>
-      <c r="C14" s="3" t="inlineStr"/>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>150</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>230</v>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Venus V.B</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Copa Retro</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr"/>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Pegada</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="n">
-        <v>180</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>220</v>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Mod II Agua</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Copa Premium Mediana</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr"/>
-      <c r="C16" s="3" t="inlineStr"/>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="n">
-        <v>230</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>220</v>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Mini Marisco</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Copa Premium Chica</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr"/>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="n">
-        <v>220</v>
-      </c>
-      <c r="F17" s="3" t="n">
-        <v>220</v>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Mod II Agua</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Copa Silvia Agua</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr"/>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Pegada</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="n">
-        <v>180</v>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>220</v>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Silvia Agua</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K18" s="3" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Separar corte caliente (c/c) y c/ en la pestaña COPAS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -1117,20 +1117,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1151,40 +1152,45 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Medida (℅)</t>
+          <t>Corte caliente (c/c)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>c/</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Pie</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Nota en lápiz</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1207,27 +1213,28 @@
           <t>15,3</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Lorena V.B</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="K2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1238,27 +1245,28 @@
       <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="K3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1269,27 +1277,28 @@
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Presi V.T</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="K4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1308,27 +1317,28 @@
           <t>19,7</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n">
-        <v>220</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="3" t="n">
         <v>220</v>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>London 98</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="K5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>El peso está remarcado/sobrescrito: confirmar que es 220</t>
         </is>
@@ -1351,27 +1361,28 @@
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="n">
         <v>250</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>London 98</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="K6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1386,27 +1397,28 @@
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="n">
         <v>230</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="G7" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>London 98</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J7" s="3" t="n">
+      <c r="K7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>El pie no está escrito: hay comillas (") debajo de "Pie London 98" de la fila de arriba</t>
         </is>
@@ -1425,27 +1437,28 @@
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Delise</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="K8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1460,23 +1473,24 @@
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>220</v>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="K9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1495,23 +1509,24 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>220</v>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="K10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1525,32 +1540,33 @@
           <t>Estirada</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="F11" s="2" t="n">
         <v>170</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="G11" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Presi Agua</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J11" s="2" t="n">
+      <c r="K11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1560,36 +1576,37 @@
       </c>
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="F12" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Venus V.B</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="K12" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1604,31 +1621,32 @@
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>220</v>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Mod II Agua</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J13" s="2" t="n">
+      <c r="K13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1639,27 +1657,28 @@
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="n">
         <v>230</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>220</v>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Mini Marisco</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="K14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1670,27 +1689,28 @@
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="n">
-        <v>220</v>
-      </c>
+      <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="n">
         <v>220</v>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Mod II Agua</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="K15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1705,31 +1725,32 @@
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="n">
         <v>180</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>220</v>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Silvia Agua</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="K16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Agregar copas de la foto 3 (pinza, molde, destino)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -1117,21 +1117,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="55" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1152,7 +1155,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Corte caliente (c/c)</t>
+          <t>Corte caliente c/c (altura)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1177,20 +1180,35 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Pinza</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Molde</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Destino</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Nota en lápiz</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1226,15 +1244,18 @@
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="N2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1253,20 +1274,23 @@
         <v>200</v>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="N3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1290,15 +1314,18 @@
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="N4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1330,15 +1357,18 @@
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="N5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>El peso está remarcado/sobrescrito: confirmar que es 220</t>
         </is>
@@ -1374,15 +1404,18 @@
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="N6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1410,15 +1443,18 @@
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K7" s="3" t="n">
+      <c r="N7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>El pie no está escrito: hay comillas (") debajo de "Pie London 98" de la fila de arriba</t>
         </is>
@@ -1450,15 +1486,18 @@
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="N8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1482,15 +1521,18 @@
       </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="N9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1518,15 +1560,18 @@
       </c>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="N10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1558,15 +1603,18 @@
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="N11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1593,20 +1641,23 @@
           <t>Venus V.B</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="N12" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1633,20 +1684,23 @@
           <t>Mod II Agua</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="N13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1670,15 +1724,18 @@
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="N14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1702,15 +1759,18 @@
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="N15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1737,20 +1797,387 @@
           <t>Silvia Agua</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="N16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Copa Expresión</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Copa Martini Champ</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>C. Ruiz</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Eva Champ</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Copa Nueva Progreso</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>21,0</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Copa Hurricane</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>20,5</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Coñac London 98</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr"/>
+      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>Pinza: se lee 90 (las demás dicen 19). Confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Copa Patagonia Cerveza</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>15,3</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>London 98</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Copa Taby Cerveza</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>14,3</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Venus Agua</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Copa Ani</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>G / German</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Pegada (pierna fina)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Marisco Deisy</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Copa "G"</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>German</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>Molde copa "G": puede ser G o 6. Confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Copa Checo Flauta</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Estirada</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>22,0</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>170</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Presi Agua</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Erika de Rosemblet</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Agregar tarros y floreros de la foto 4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -2190,16 +2190,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2215,29 +2218,296 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Capacidad</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Corte caliente c/c (altura)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Nota en lápiz</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Florero Cónico</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>1 L</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>14,5</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>900</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Florero Cónico</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2 L</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>18,0</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Florero 12x30</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>30,0</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Florero 17x50</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>47,0</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Florero 17x50 2 cortes</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Florero Lila</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>15,3</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>650</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Chico</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Florero Lila Diagonal</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Diagonal</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>850</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Dice "c/c Diagonal" sin altura: ¿corte en diagonal?</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Florero Potiche</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>23,5</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2430,16 +2700,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2455,29 +2728,304 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Capacidad</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Corte caliente c/c (altura)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Nota en lápiz</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Tarro Cónico</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>1/2 L</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>13,0</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Tarro Claret</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>1 1/2 L</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>20,1</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>B:55</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Tiene un segundo "B:55" al final del renglón. ¿Qué es?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Tarro Bocha</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>3/4 L</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>11,0</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Tarro M-13x8,5</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>8,5</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Tarro M-13x15</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>15,0</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Tarro M-13x20</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>20,0</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Tarro M-13x25</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>25,0</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Tarro M-13x30</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>30,0</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Agregar floreros, tulipas, pamelas y botellones de la foto 5
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -2190,7 +2190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2199,10 +2199,11 @@
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2228,30 +2229,35 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Otro corte</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Nota en lápiz</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -2274,22 +2280,23 @@
           <t>14,5</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="n">
         <v>900</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>150</v>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Sin título</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="J2" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2308,22 +2315,23 @@
           <t>18,0</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="n">
         <v>1000</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Sin título</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="J3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2338,22 +2346,23 @@
           <t>30,0</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="n">
         <v>1000</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Sin título</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="J4" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2368,22 +2377,23 @@
           <t>47,0</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="n">
         <v>2500</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Sin título</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="J5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2394,22 +2404,27 @@
       <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2 cortes</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
         <v>3000</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Sin título</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="J6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2424,26 +2439,27 @@
           <t>15,3</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="n">
         <v>650</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Chico</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Sin título</t>
         </is>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="J7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2458,22 +2474,23 @@
           <t>Diagonal</t>
         </is>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="n">
         <v>850</v>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="G8" s="3" t="n">
         <v>150</v>
       </c>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Sin título</t>
         </is>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="J8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>Dice "c/c Diagonal" sin altura: ¿corte en diagonal?</t>
         </is>
@@ -2492,22 +2509,155 @@
           <t>23,5</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="n">
         <v>1200</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>120</v>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Sin título</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="J9" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Florero Cuadrado Grande</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Florero Mod 11</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Cenatiempo</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>26,5</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>c/ 24 cm</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>700</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Abajo dice: corte c/24cm "Cenatiempo". Confirmar cómo se escribe Cenatiempo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Florero Cónico Alto</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>28,0</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Florero Cónico Bajo</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>19,3</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2520,16 +2670,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2545,29 +2696,86 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Corte caliente c/c (altura)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Tulipa Mini Mum</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
+        <v>900</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Tulipa Rochester</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>20,5</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2580,16 +2788,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2605,29 +2814,142 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Corte caliente c/c (altura)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Pamela x21</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>9,0</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Pamela x16</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>7,6</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Pamela x11</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Pamela x10</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>5,3</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2640,16 +2962,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2665,29 +2988,106 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Corte caliente c/c (altura)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Botellón Neo</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Botellón Inti Chico</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Botellón Mini</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Agregar centros, tapas, botellones, jarra y aceitera de la foto 6
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -18,7 +18,8 @@
     <sheet name="TAPA" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="JARRA" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="ACEITERA" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="PRENSA" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="OTROS" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="PRENSA" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -531,16 +532,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -556,29 +558,62 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Corte caliente c/c (altura)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Jarra Carafe con Pico y Asa</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>16,0</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -591,16 +626,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -616,29 +652,58 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Corte caliente c/c (altura)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Aceitera Cónico Chico con Pico</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -646,6 +711,104 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre entre comillas</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Corte caliente c/c (altura)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Peso (P)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Base (B)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Sección del cuaderno</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Foto Nº</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Bombe Gigante</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>15,8</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>700</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>No entra en ninguna categoría. ¿Dónde va?</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2962,7 +3125,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3088,6 +3251,86 @@
         <v>5</v>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Botellón Decanter</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Botellón Decantador Progreso</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Escrito en lápiz debajo del Botellón Decanter. ¿Es la misma pieza con otro nombre?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Botellón Nahuel</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Escrito en lápiz</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3438,16 +3681,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -3463,29 +3707,86 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Corte caliente c/c (altura)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Centro Oreford Grande</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
+        <v>2800</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Centro Porta Vela</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>9,5</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3498,16 +3799,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -3523,27 +3826,186 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Corte caliente c/c (altura)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Peso (P)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Base (B)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Molde</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Tapa Quesera 1/2 Esfera</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>c/c (sin altura)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Dice c/c pero no tiene la altura</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Tapa Quesera con Botón</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Tapa 17x20</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>20,0</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Tapa 17x13</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>13,0</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Tapa M-13</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Also</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Sin título</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Molde: se lee "Also". Confirmar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar copas de la foto 7
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -1280,7 +1280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2341,6 +2341,642 @@
         <v>3</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Copa Premium Borgoña</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Copa Premium Borgoña R</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>R / C. Ruiz</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H26" s="3" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr"/>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>Renglón con comillas de repetición debajo de Premium Borgoña, con "R" y "C. Ruiz". ¿Es otra versión de la misma copa?</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Copa G</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="n">
+        <v>260</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>230</v>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Andrea Agua</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr"/>
+      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr"/>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>¿Es la misma copa "G" que figura como molde de la Copa Ani (foto 3)?</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Copa Beefeater</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Copa Bordeau Agua</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>7x7 Champ</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Copa H</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Mod II Agua</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Copa Cabernet</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Copa Terraza</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Cheval</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr"/>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Cheval</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr"/>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="O32" s="3" t="inlineStr">
+        <is>
+          <t>La pierna tiene comillas de repetición (") debajo de "P.Peg" de la Cabernet. "Molde Cheval" está en lápiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Copa 2 Tiempo</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Clásica</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Copa Alma</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr"/>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr"/>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>Dice "Pie" pero no está escrito cuál</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Copa Degustación</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="n">
+        <v>150</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Copa M-H Vino</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>M-H</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>London 98</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>C. Ruiz</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Copa Vitalia</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Clásica</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Copa Vinarte</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr"/>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Alta y Pegada</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr"/>
+      <c r="F38" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Presi Vino Tinto</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr"/>
+      <c r="J38" s="3" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>Dice "P.Alta" y "P.Peg" a la vez</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Copa Soire Flauta</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>220</v>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Presi Agua</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Copa Brunelo Vino</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Pegada</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Brenda Agua</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O40" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Pasar los nombres entre comillas o en lápiz a una columna Cliente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -470,7 +470,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -487,7 +487,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -536,7 +536,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -553,7 +553,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -630,7 +630,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -647,7 +647,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -720,7 +720,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -737,7 +737,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -819,7 +819,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -840,7 +840,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -1209,14 +1209,10 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Vidrio</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>U</t>
-        </is>
-      </c>
+          <t>Vidrio U</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="n">
         <v>620</v>
       </c>
@@ -1280,11 +1276,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O40"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -1293,11 +1289,9 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="55" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1308,7 +1302,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1353,25 +1347,15 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Destino</t>
+          <t>Sección del cuaderno</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Nota en lápiz</t>
+          <t>Foto Nº</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Sección del cuaderno</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Foto Nº</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1408,17 +1392,15 @@
       </c>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N2" s="2" t="n">
+      <c r="L2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1426,7 +1408,11 @@
           <t>Copa Presidente Champ</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
@@ -1439,21 +1425,15 @@
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N3" s="2" t="n">
+      <c r="L3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1478,17 +1458,15 @@
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n">
+      <c r="L4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1521,17 +1499,15 @@
       </c>
       <c r="I5" s="3" t="inlineStr"/>
       <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>El peso está remarcado/sobrescrito: confirmar que es 220</t>
         </is>
@@ -1540,14 +1516,10 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Copa Barón</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>Copa Barón B</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Estirada</t>
@@ -1568,17 +1540,15 @@
       </c>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n">
+      <c r="L6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1607,17 +1577,15 @@
       </c>
       <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="N7" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>El pie no está escrito: hay comillas (") debajo de "Pie London 98" de la fila de arriba</t>
         </is>
@@ -1650,17 +1618,15 @@
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n">
+      <c r="L8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1685,17 +1651,15 @@
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="L9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1724,17 +1688,15 @@
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N10" s="2" t="n">
+      <c r="L10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1767,17 +1729,15 @@
       </c>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n">
+      <c r="L11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1785,7 +1745,11 @@
           <t>Copa Him-Chan Agua</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
@@ -1806,21 +1770,15 @@
       </c>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n">
+      <c r="L12" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1828,7 +1786,11 @@
           <t>Copa Retro</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Pegada</t>
@@ -1849,21 +1811,15 @@
       </c>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="L13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1888,17 +1844,15 @@
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N14" s="2" t="n">
+      <c r="L14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1923,17 +1877,15 @@
       </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N15" s="2" t="n">
+      <c r="L15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1941,7 +1893,11 @@
           <t>Copa Silvia Agua</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Pegada</t>
@@ -1962,21 +1918,15 @@
       </c>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N16" s="2" t="n">
+      <c r="L16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2005,17 +1955,15 @@
       </c>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N17" s="2" t="n">
+      <c r="L17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2048,17 +1996,15 @@
       </c>
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N18" s="2" t="n">
+      <c r="L18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2091,17 +2037,15 @@
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N19" s="2" t="n">
+      <c r="L19" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -2134,17 +2078,15 @@
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr"/>
-      <c r="K20" s="3" t="inlineStr"/>
-      <c r="L20" s="3" t="inlineStr"/>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="M20" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="N20" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="O20" s="3" t="inlineStr">
         <is>
           <t>Pinza: se lee 90 (las demás dicen 19). Confirmar</t>
         </is>
@@ -2181,17 +2123,15 @@
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N21" s="2" t="n">
+      <c r="L21" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2224,17 +2164,15 @@
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N22" s="2" t="n">
+      <c r="L22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -2244,7 +2182,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>G / German</t>
+          <t>German</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -2273,21 +2211,15 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>German</t>
-        </is>
-      </c>
-      <c r="L23" s="3" t="inlineStr"/>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>3</v>
+      </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="N23" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="O23" s="3" t="inlineStr">
-        <is>
-          <t>Molde copa "G": puede ser G o 6. Confirmar</t>
+          <t>Molde copa "G": puede ser G o 6. Confirmar En el cuaderno dice Destino: "German".</t>
         </is>
       </c>
     </row>
@@ -2330,17 +2262,15 @@
           <t>Erika de Rosemblet</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N24" s="2" t="n">
+      <c r="L24" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="O24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2361,17 +2291,15 @@
       <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N25" s="2" t="n">
+      <c r="L25" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -2381,7 +2309,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>R / C. Ruiz</t>
+          <t>C. Ruiz</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
@@ -2396,17 +2324,15 @@
       <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr"/>
       <c r="J26" s="3" t="inlineStr"/>
-      <c r="K26" s="3" t="inlineStr"/>
-      <c r="L26" s="3" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="n">
+        <v>7</v>
+      </c>
       <c r="M26" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="N26" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="O26" s="3" t="inlineStr">
         <is>
           <t>Renglón con comillas de repetición debajo de Premium Borgoña, con "R" y "C. Ruiz". ¿Es otra versión de la misma copa?</t>
         </is>
@@ -2418,11 +2344,7 @@
           <t>Copa G</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
+      <c r="B27" s="3" t="inlineStr"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Pegada</t>
@@ -2443,17 +2365,15 @@
       </c>
       <c r="I27" s="3" t="inlineStr"/>
       <c r="J27" s="3" t="inlineStr"/>
-      <c r="K27" s="3" t="inlineStr"/>
-      <c r="L27" s="3" t="inlineStr"/>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="n">
+        <v>7</v>
+      </c>
       <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="N27" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="O27" s="3" t="inlineStr">
         <is>
           <t>¿Es la misma copa "G" que figura como molde de la Copa Ani (foto 3)?</t>
         </is>
@@ -2482,17 +2402,15 @@
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N28" s="2" t="n">
+      <c r="L28" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2517,17 +2435,15 @@
       </c>
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N29" s="2" t="n">
+      <c r="L29" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2537,7 +2453,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>Renato</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2560,21 +2476,15 @@
       </c>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N30" s="2" t="n">
+      <c r="L30" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2599,17 +2509,15 @@
       <c r="H31" s="2" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N31" s="2" t="n">
+      <c r="L31" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -2642,17 +2550,15 @@
           <t>Cheval</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr"/>
-      <c r="L32" s="3" t="inlineStr"/>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="n">
+        <v>7</v>
+      </c>
       <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="O32" s="3" t="inlineStr">
         <is>
           <t>La pierna tiene comillas de repetición (") debajo de "P.Peg" de la Cabernet. "Molde Cheval" está en lápiz</t>
         </is>
@@ -2681,17 +2587,15 @@
       </c>
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N33" s="2" t="n">
+      <c r="L33" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -2716,17 +2620,15 @@
       <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr"/>
       <c r="J34" s="3" t="inlineStr"/>
-      <c r="K34" s="3" t="inlineStr"/>
-      <c r="L34" s="3" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="n">
+        <v>7</v>
+      </c>
       <c r="M34" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="N34" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="O34" s="3" t="inlineStr">
         <is>
           <t>Dice "Pie" pero no está escrito cuál</t>
         </is>
@@ -2751,17 +2653,15 @@
       <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr"/>
-      <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr"/>
-      <c r="M35" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N35" s="2" t="n">
+      <c r="L35" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2771,7 +2671,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>M-H</t>
+          <t>C. Ruiz</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2794,21 +2694,15 @@
       </c>
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>C. Ruiz</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N36" s="2" t="n">
+      <c r="L36" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2816,7 +2710,11 @@
           <t>Copa Vitalia</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Pegada</t>
@@ -2837,21 +2735,15 @@
       </c>
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N37" s="2" t="n">
+      <c r="L37" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2859,7 +2751,11 @@
           <t>Copa Vinarte</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr"/>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Alta y Pegada</t>
@@ -2880,21 +2776,15 @@
       </c>
       <c r="I38" s="3" t="inlineStr"/>
       <c r="J38" s="3" t="inlineStr"/>
-      <c r="K38" s="3" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Copas</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="n">
+        <v>7</v>
       </c>
       <c r="M38" s="3" t="inlineStr">
-        <is>
-          <t>Copas</t>
-        </is>
-      </c>
-      <c r="N38" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="O38" s="3" t="inlineStr">
         <is>
           <t>Dice "P.Alta" y "P.Peg" a la vez</t>
         </is>
@@ -2927,17 +2817,15 @@
       </c>
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr"/>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N39" s="2" t="n">
+      <c r="L39" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2966,17 +2854,15 @@
       </c>
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="N40" s="2" t="n">
+      <c r="L40" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="O40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2993,7 +2879,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -3013,7 +2899,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3473,7 +3359,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -3490,7 +3376,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3591,7 +3477,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -3608,7 +3494,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3765,7 +3651,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -3782,7 +3668,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3983,7 +3869,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -4002,7 +3888,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -4321,7 +4207,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -4338,7 +4224,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -4439,7 +4325,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -4457,7 +4343,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nombre entre comillas</t>
+          <t>Cliente</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Revert "Pasar los nombres entre comillas o en lápiz a una columna Cliente"
This reverts commit f7a1ada5dae745b0411c308e7653c37f090b2a3e.
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -470,7 +470,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -487,7 +487,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -536,7 +536,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -553,7 +553,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -630,7 +630,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -647,7 +647,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -720,7 +720,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -737,7 +737,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -819,7 +819,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -840,7 +840,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -1209,10 +1209,14 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Vidrio U</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr"/>
+          <t>Vidrio</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
       <c r="D13" s="3" t="n">
         <v>620</v>
       </c>
@@ -1276,11 +1280,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -1289,9 +1293,11 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="55" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="55" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1302,7 +1308,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -1347,15 +1353,25 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Destino</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Nota en lápiz</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1392,15 +1408,17 @@
       </c>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="N2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1408,11 +1426,7 @@
           <t>Copa Presidente Champ</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
+      <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
@@ -1425,15 +1439,21 @@
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="N3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1458,15 +1478,17 @@
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="N4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1499,15 +1521,17 @@
       </c>
       <c r="I5" s="3" t="inlineStr"/>
       <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L5" s="3" t="n">
+      <c r="N5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>El peso está remarcado/sobrescrito: confirmar que es 220</t>
         </is>
@@ -1516,10 +1540,14 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Copa Barón B</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr"/>
+          <t>Copa Barón</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Estirada</t>
@@ -1540,15 +1568,17 @@
       </c>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L6" s="2" t="n">
+      <c r="N6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1577,15 +1607,17 @@
       </c>
       <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L7" s="3" t="n">
+      <c r="N7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>El pie no está escrito: hay comillas (") debajo de "Pie London 98" de la fila de arriba</t>
         </is>
@@ -1618,15 +1650,17 @@
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L8" s="2" t="n">
+      <c r="N8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1651,15 +1685,17 @@
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="N9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1688,15 +1724,17 @@
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L10" s="2" t="n">
+      <c r="N10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1729,15 +1767,17 @@
       </c>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L11" s="2" t="n">
+      <c r="N11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1745,11 +1785,7 @@
           <t>Copa Him-Chan Agua</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
+      <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr">
@@ -1770,15 +1806,21 @@
       </c>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L12" s="2" t="n">
+      <c r="N12" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1786,11 +1828,7 @@
           <t>Copa Retro</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
+      <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Pegada</t>
@@ -1811,15 +1849,21 @@
       </c>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L13" s="2" t="n">
+      <c r="N13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1844,15 +1888,17 @@
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L14" s="2" t="n">
+      <c r="N14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1877,15 +1923,17 @@
       </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L15" s="2" t="n">
+      <c r="N15" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1893,11 +1941,7 @@
           <t>Copa Silvia Agua</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
+      <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Pegada</t>
@@ -1918,15 +1962,21 @@
       </c>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L16" s="2" t="n">
+      <c r="N16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1955,15 +2005,17 @@
       </c>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L17" s="2" t="n">
+      <c r="N17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1996,15 +2048,17 @@
       </c>
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L18" s="2" t="n">
+      <c r="N18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2037,15 +2091,17 @@
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L19" s="2" t="n">
+      <c r="N19" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -2078,15 +2134,17 @@
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr"/>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L20" s="3" t="n">
+      <c r="N20" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="O20" s="3" t="inlineStr">
         <is>
           <t>Pinza: se lee 90 (las demás dicen 19). Confirmar</t>
         </is>
@@ -2123,15 +2181,17 @@
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L21" s="2" t="n">
+      <c r="N21" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2164,15 +2224,17 @@
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L22" s="2" t="n">
+      <c r="N22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -2182,7 +2244,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>German</t>
+          <t>G / German</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -2211,15 +2273,21 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
+          <t>German</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L23" s="3" t="n">
+      <c r="N23" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="M23" s="3" t="inlineStr">
-        <is>
-          <t>Molde copa "G": puede ser G o 6. Confirmar En el cuaderno dice Destino: "German".</t>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>Molde copa "G": puede ser G o 6. Confirmar</t>
         </is>
       </c>
     </row>
@@ -2262,15 +2330,17 @@
           <t>Erika de Rosemblet</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L24" s="2" t="n">
+      <c r="N24" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2291,15 +2361,17 @@
       <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L25" s="2" t="n">
+      <c r="N25" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -2309,7 +2381,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>C. Ruiz</t>
+          <t>R / C. Ruiz</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
@@ -2324,15 +2396,17 @@
       <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr"/>
       <c r="J26" s="3" t="inlineStr"/>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr"/>
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L26" s="3" t="n">
+      <c r="N26" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="O26" s="3" t="inlineStr">
         <is>
           <t>Renglón con comillas de repetición debajo de Premium Borgoña, con "R" y "C. Ruiz". ¿Es otra versión de la misma copa?</t>
         </is>
@@ -2344,7 +2418,11 @@
           <t>Copa G</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Pegada</t>
@@ -2365,15 +2443,17 @@
       </c>
       <c r="I27" s="3" t="inlineStr"/>
       <c r="J27" s="3" t="inlineStr"/>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr"/>
+      <c r="M27" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L27" s="3" t="n">
+      <c r="N27" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="M27" s="3" t="inlineStr">
+      <c r="O27" s="3" t="inlineStr">
         <is>
           <t>¿Es la misma copa "G" que figura como molde de la Copa Ani (foto 3)?</t>
         </is>
@@ -2402,15 +2482,17 @@
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L28" s="2" t="n">
+      <c r="N28" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2435,15 +2517,17 @@
       </c>
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L29" s="2" t="n">
+      <c r="N29" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2453,7 +2537,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Renato</t>
+          <t>H</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2476,15 +2560,21 @@
       </c>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L30" s="2" t="n">
+      <c r="N30" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2509,15 +2599,17 @@
       <c r="H31" s="2" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L31" s="2" t="n">
+      <c r="N31" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -2550,15 +2642,17 @@
           <t>Cheval</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="K32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr"/>
+      <c r="M32" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L32" s="3" t="n">
+      <c r="N32" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="M32" s="3" t="inlineStr">
+      <c r="O32" s="3" t="inlineStr">
         <is>
           <t>La pierna tiene comillas de repetición (") debajo de "P.Peg" de la Cabernet. "Molde Cheval" está en lápiz</t>
         </is>
@@ -2587,15 +2681,17 @@
       </c>
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L33" s="2" t="n">
+      <c r="N33" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -2620,15 +2716,17 @@
       <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr"/>
       <c r="J34" s="3" t="inlineStr"/>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="K34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr"/>
+      <c r="M34" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L34" s="3" t="n">
+      <c r="N34" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="M34" s="3" t="inlineStr">
+      <c r="O34" s="3" t="inlineStr">
         <is>
           <t>Dice "Pie" pero no está escrito cuál</t>
         </is>
@@ -2653,15 +2751,17 @@
       <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr"/>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L35" s="2" t="n">
+      <c r="N35" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2671,7 +2771,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>C. Ruiz</t>
+          <t>M-H</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2694,15 +2794,21 @@
       </c>
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>C. Ruiz</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L36" s="2" t="n">
+      <c r="N36" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2710,11 +2816,7 @@
           <t>Copa Vitalia</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
+      <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Pegada</t>
@@ -2735,15 +2837,21 @@
       </c>
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L37" s="2" t="n">
+      <c r="N37" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2751,11 +2859,7 @@
           <t>Copa Vinarte</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
+      <c r="B38" s="3" t="inlineStr"/>
       <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Alta y Pegada</t>
@@ -2776,15 +2880,21 @@
       </c>
       <c r="I38" s="3" t="inlineStr"/>
       <c r="J38" s="3" t="inlineStr"/>
-      <c r="K38" s="3" t="inlineStr">
+      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L38" s="3" t="n">
+      <c r="N38" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="M38" s="3" t="inlineStr">
+      <c r="O38" s="3" t="inlineStr">
         <is>
           <t>Dice "P.Alta" y "P.Peg" a la vez</t>
         </is>
@@ -2817,15 +2927,17 @@
       </c>
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L39" s="2" t="n">
+      <c r="N39" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2854,15 +2966,17 @@
       </c>
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>Copas</t>
         </is>
       </c>
-      <c r="L40" s="2" t="n">
+      <c r="N40" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="M40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2879,7 +2993,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -2899,7 +3013,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3359,7 +3473,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -3376,7 +3490,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3477,7 +3591,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -3494,7 +3608,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3651,7 +3765,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -3668,7 +3782,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3869,7 +3983,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -3888,7 +4002,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -4207,7 +4321,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -4224,7 +4338,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -4325,7 +4439,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -4343,7 +4457,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Nombre entre comillas</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Agregar vasos de la foto 8
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -466,17 +466,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -492,7 +495,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Altura</t>
+          <t>Altura (c/c Alt)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -507,17 +510,448 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Boca</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Molde</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Sección del cuaderno</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Foto Nº</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Splendid Vino</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Gastro Baires</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Vaso IPA Cerveza</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>18,3</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Vaso IPA</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Vaso Whisky A</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>A / Raye</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>12,8</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>480</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Las comillas abarcan "A" y "Raye": ¿es "A" el modelo y "Raye" otro nombre? La altura puede ser 12,8</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Nico R Vino</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="n">
+        <v>370</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>C. Ruiz</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Cerveza Bajo</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>15,3</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Vaso D-F 2</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>16,7</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Terrario 10x8 con Asa</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>c/c (sin altura)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Andrea Borgoña</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Está en la hoja de Vasos. Dice c/c pero sin altura</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Globo x16</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>c/c (sin altura)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>700</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Globo x15</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Está en la hoja de Vasos. Dice c/c pero sin altura</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Globo x8 con Cuello</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>A Placa</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Está en la hoja de Vasos</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Botella Cairel</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Calentar molde</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Está en la hoja de Vasos. "Calentar molde" (en lápiz) está entre Botella y Globo Cairel: ¿para cuál es?</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Globo Cairel</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Rococo</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Está en la hoja de Vasos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar vasos de la foto 9
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -954,6 +954,488 @@
           <t>Está en la hoja de Vasos</t>
         </is>
       </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Vaso 9x9 F. Liso</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Vaso 8,5x8,5 F. Liso</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Vaso 7x7 F. Liso</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Vaso Pipetua</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="n">
+        <v>470</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Confirmar el nombre: se lee "Pipetua"</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Recto T. Largo</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="n">
+        <v>480</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Barrilito</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Bombe</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Vaso Bombe Fondo Hueco</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>En lápiz, con comillas de repetición debajo del Vaso Bombe. No tiene peso; la base tiene un número tachado y 300</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Cónico B-R</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Maracaná</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>20,0</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Fernet Progreso</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>18,0</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Antares Nº 2</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>14,4</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Temple</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>21,2</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>470</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Maxi</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Hilton Agua</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>11,0</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Hilton Jugo</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Chivas</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>10,5</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Tapin Cerveza</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>21,0</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>De Rivas</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Vasos</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Agregar vasos, tulipa y tapa de la foto 10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdfmV2wNEqdhzbLzVzpHMK
</commit_message>
<xml_diff>
--- a/planilla/planilla_piezas.xlsx
+++ b/planilla/planilla_piezas.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1178,31 +1178,39 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Vaso Cónico B-R</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr"/>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="n">
+      <c r="B22" s="3" t="inlineStr"/>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>14,3</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
         <v>380</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="3" t="n">
         <v>280</v>
       </c>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Vasos</t>
         </is>
       </c>
-      <c r="J22" s="2" t="n">
+      <c r="J22" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Aparece otra vez en la foto 10 con los mismos números y c/c 14,3 (la altura sale de ahí)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1436,6 +1444,553 @@
         <v>9</v>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Vaso Cónico B-R (2ª versión)</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr"/>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>En lápiz, con comillas de repetición debajo del Vaso Cónico B-R</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Té</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Vaso Nico Vino</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F32" s="3" t="inlineStr"/>
+      <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Distinto del "Vaso Nico R Vino" (P:370) de la foto 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Danés Licor</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Danés Whisky</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="n">
+        <v>650</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Luz</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>5,6</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>A Placa</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Violetero Faena</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr"/>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>12,0</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="F36" s="3" t="inlineStr"/>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>No es vaso pero está en la lista de vasos</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Carafe</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>7,3</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Con talón</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Botella</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>14,5</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Vaso Lata</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr"/>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>14,0</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>330</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F39" s="3" t="inlineStr"/>
+      <c r="G39" s="3" t="inlineStr"/>
+      <c r="H39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>La altura 13,8 está tachada y corregida a 14,0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Cid</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>7,5</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Botín</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>18,0</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Vaso Popo Gigante</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr"/>
+      <c r="C42" s="3" t="inlineStr"/>
+      <c r="D42" s="3" t="n">
+        <v>116</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="F42" s="3" t="inlineStr"/>
+      <c r="G42" s="3" t="inlineStr"/>
+      <c r="H42" s="3" t="inlineStr"/>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>Peso 116: confirmar (es bajo para un vaso gigante)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Vaso Whisky C</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Vaso Whisky C Desfondado</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>C / Renato</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr"/>
+      <c r="D44" s="3" t="n">
+        <v>260</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F44" s="3" t="inlineStr"/>
+      <c r="G44" s="3" t="inlineStr"/>
+      <c r="H44" s="3" t="inlineStr"/>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>El peso está sobrescrito: confirmar 260</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Vaso Recto Whisky</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr"/>
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="F45" s="3" t="inlineStr"/>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>c/14</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Dice "c/14" (igual que en algunas copas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Vaso Petit</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr"/>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>4,5</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F46" s="3" t="inlineStr"/>
+      <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>A Placa</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>Debajo del P:120 hay un "150" en lápiz. La altura dice "Alt: 4,5" sin c/c</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4385,7 +4940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4491,6 +5046,34 @@
         <v>5</v>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tulipa Difusa</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Está en la lista de vasos</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5351,7 +5934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5561,6 +6144,39 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Tapa 995</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>13,0</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>280</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Sin título (sigue Vasos)</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Está en la lista de vasos</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>